<commit_message>
feat: scope support agents to their assigned projects (decision I)
Agents now see only tickets for the client companies they cover (new
AGENT_COMPANIES bridge table) instead of every client's open queue.
The 4 roles are unchanged: Manager, L1/L2/L3 tiers, and Project Lead
are NOT separate roles (overseer behaviour, Escalate action, and a
deferred is_lead flag respectively).

Synced across every artifact: brief, visual HTML, kickoff deck,
requirements tracker, page-build-guide (7-table schema + AGENT_COMPANIES,
the visibility predicate in all 5 places, and the Page 10a admin grid),
CLAUDE.md, and the tenant-isolation-auditor agent.
</commit_message>
<xml_diff>
--- a/docs/Ticketing-Requirements.xlsx
+++ b/docs/Ticketing-Requirements.xlsx
@@ -2338,7 +2338,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="25" t="inlineStr">
         <is>
@@ -2599,7 +2598,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Tickets assigned to them + open queue</t>
+          <t>Tickets for their assigned projects only (clients they cover) - never clients they are not on</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -2644,7 +2643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2830,6 +2829,28 @@
       </c>
       <c r="D11" s="5" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Agents see every client, or only the projects they are assigned to?</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Scoped to assigned projects (AGENT_COMPANIES join)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>CONFIRMED: agents scoped to their projects; 4 roles kept (Manager=overseer not a role, L1/L2/L3=Escalate no level field, Project Lead deferred as is_lead flag)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
docs: add ticket aging (stale/overdue) build recipe + sync project docs
- page-build-guide: new 'Ticket aging' add-on section (stale flag + overdue
  highlight) with role-aware §A.7 predicate, declarative IR highlight steps,
  CSS, and per-role isolation tests; reviewed by tenant-isolation-auditor
- page-build-guide: align *_AT/SLA_DUE columns to TIMESTAMP WITH LOCAL TIME ZONE
- brief: add timestamps & history-vocabulary convention (enables aging/FRT
  metrics with no schema change); fix reopen-detection note
- include pre-existing doc/tooling updates (READMEs, deck/sheet, sync-docs)
</commit_message>
<xml_diff>
--- a/docs/Ticketing-Requirements.xlsx
+++ b/docs/Ticketing-Requirements.xlsx
@@ -1543,12 +1543,12 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Stretch</t>
+          <t>Tickets - Stretch</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>File attachments on tickets.</t>
+          <t>File / screenshot attachments on a ticket (proof/evidence); stored in TICKET_ATTACHMENTS, tenant-scoped (brief §5.1).</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -2416,6 +2416,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: sync all artifacts — severity/priority split, SLA→SHOULD, decisions J/K, client assign
Promote SLA breach highlighting from COULD to SHOULD (9 total), add
decisions J (clients assign agents) and K (severity ≠ priority), update
FR-7/10/15/23, data model (8 tables with SLA_TARGETS), roles, and mockups.
All artifacts verified consistent with the brief.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Ticketing-Requirements.xlsx
+++ b/docs/Ticketing-Requirements.xlsx
@@ -581,6 +581,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -859,12 +860,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Tickets - Core</t>
+          <t>Tickets</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>A client can raise a ticket (subject, description, category, priority).</t>
+          <t>A client can raise a ticket (subject, description, category, severity). Severity (business impact) is client-set; Priority (work order) is support-set.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -973,12 +974,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Tickets - Core</t>
+          <t>Tickets</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>System Admin can assign / reassign a ticket to a support agent.</t>
+          <t>A ticket can be assigned/reassigned to a support agent. System Admin assigns anyone; clients assign from agents mapped to their company; agents self-assign.</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -1168,7 +1169,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>See a list of all permitted tickets, filterable by status, priority, company, assignee.</t>
+          <t>See a list of permitted tickets, filterable by status, priority, severity, company, assignee. Includes ticket age column and SLA breach indicator.</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1467,12 +1468,12 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Stretch</t>
+          <t>SLA &amp; Aging</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>SLA target per priority with breach highlighting.</t>
+          <t>SLA target per severity with breach highlighting — global SLA_TARGETS table, colour-coded indicators (no timers).</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -1482,7 +1483,7 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>COULD</t>
+          <t>SHOULD</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -2416,7 +2417,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
docs: ITIL 4 alignment — reframe as production system, add FRs 30–34, add itil-advisor agent
Reframe project from hackathon prototype to production system (demo 16 Jul 2026).
Adopt ITIL 4 Incident + Service Request Management as guiding framework.
Add 5 ITIL-driven SHOULDs (ticket type, first-response tracking, SLA compliance
KPI, workload LOV, severity guidance), promote FR-22 to SHOULD, rename severity
Cosmetic→Low, reorganize FUTURE into ITIL P1–P4 production roadmap.
New itil-advisor agent for ongoing ITIL alignment review.
Scope: MUST=17, SHOULD=15, COULD=2. All artifacts synced and verified.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Ticketing-Requirements.xlsx
+++ b/docs/Ticketing-Requirements.xlsx
@@ -554,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1435,7 +1434,7 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>When a client's ticket changes status, they are notified.</t>
+          <t>When a client's ticket changes status, they are notified via email (ITIL: communication at every lifecycle touchpoint).</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -1445,7 +1444,7 @@
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>COULD</t>
+          <t>SHOULD</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -1739,6 +1738,116 @@
       <c r="H33" s="8" t="inlineStr">
         <is>
           <t>APEX_MAIL.SEND on an after-insert process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>FR-30</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ITIL Alignment</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Each ticket has a ticket type: INCIDENT (break-fix) or SERVICE_REQUEST (pre-defined request). ITIL foundational distinction.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>FR-31</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ITIL Alignment</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>First-response time tracking — first_response_at timestamp + response SLA breach indicator.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>FR-32</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ITIL Alignment</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Dashboard SLA Compliance % KPI card (resolved within SLA / total resolved). The #1 ITIL metric.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>FR-33</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ITIL Alignment</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Assignment LOV shows each agent's open ticket count (workload visibility for load-balancing).</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>FR-34</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ITIL Alignment</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Create Ticket form shows severity guidance text to reduce severity inflation.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
         </is>
       </c>
     </row>
@@ -2417,6 +2526,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2461,7 +2571,7 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -2476,7 +2586,7 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -2487,7 +2597,7 @@
       </c>
       <c r="B7" s="13" t="n"/>
       <c r="C7" s="18" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: manager feedback — L1-L4 tiers, dept-scoped clients, per-company SLA, auto-escalation
5 changes from manager feedback (2026-07-02):
- Decision M: agents carry explicit L1-L4 tier (APP_USERS.tier), reversing "no level field"
- Decision L: clients assign L1 agents only (LOV filtered to tier='L1')
- Decision N: Client User sees department-scoped tickets (new DEPARTMENTS table, 9 tables)
- Decision G revised: "Reassign" = manual tier transfer (FR-26); "Escalation" = system-driven
  auto-action on SLA breach (FR-35, DBMS_SCHEDULER job) — terminology aligned with industry
- FR-23 updated: SLA per severity per company (company_id added to SLA_TARGETS)
Scope: MUST=17, SHOULD=16, COULD=2. All artifacts synced and verified.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Ticketing-Requirements.xlsx
+++ b/docs/Ticketing-Requirements.xlsx
@@ -554,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -581,6 +581,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -750,7 +751,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>A client user only sees data belonging to their own company (tenant isolation).</t>
+          <t>A client user only sees data belonging to their own company and department (tenant + dept isolation).</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -978,7 +979,7 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>A ticket can be assigned/reassigned to a support agent. System Admin assigns anyone; clients assign from agents mapped to their company; agents self-assign.</t>
+          <t>A ticket can be assigned/reassigned. System Admin assigns anyone; clients assign from L1 agents mapped to their company; agents self-assign.</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -1472,7 +1473,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>SLA target per severity with breach highlighting — global SLA_TARGETS table, colour-coded indicators (no timers).</t>
+          <t>SLA target per severity, per project (company) with breach highlighting — SLA_TARGETS keyed on (company_id, severity), colour-coded indicators.</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -1581,12 +1582,12 @@
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Tickets - Core</t>
+          <t>Tickets</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Escalate: agent/lead reassigns a ticket to a higher tier + raises priority; written to history.</t>
+          <t>A support agent/lead can reassign a ticket to a higher-tier agent (e.g. L1→L2) + optionally raise priority, written to history.</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -1846,6 +1847,28 @@
         </is>
       </c>
       <c r="E38" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>FR-35</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SLA &amp; Aging</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Auto-escalation on SLA breach — scheduled job reassigns to higher-tier agent + notifies management when SLA is at risk. System-driven.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>SHOULD</t>
         </is>
@@ -2526,7 +2549,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2571,7 +2593,7 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -2597,7 +2619,7 @@
       </c>
       <c r="B7" s="13" t="n"/>
       <c r="C7" s="18" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(mockups): sync demo with latest brief — tiers, depts, ticket types, resolve dialog, SLA page
Align the interactive mockup with all brief changes since the last sync
(manager feedback + ITIL audit). Key updates:
- Severity "Cosmetic" → "Low"; agent tiers L1–L4; department scoping
- Ticket type (Incident / Service Request) — FR-30 MUST
- Resolve dialog with resolution code + summary — FR-36
- Close dialog restricted to client/admin with inline CSAT — FR-11/FR-27
- Triage gate: priority required before In Progress — FR-37
- Per-company SLA targets with escalation_pct — FR-23/FR-35
- First-response tracking — FR-31; SLA Compliance % KPI — FR-32
- Tier-filtered escalation LOV — FR-26; severity guidance — FR-34
- New Page 13: SLA Targets management (System Admin)
- localStorage v4→v5 (reset required to pick up new seed data)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Ticketing-Requirements.xlsx
+++ b/docs/Ticketing-Requirements.xlsx
@@ -554,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1755,12 +1755,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Each ticket has a ticket type: INCIDENT (break-fix) or SERVICE_REQUEST (pre-defined request). ITIL foundational distinction.</t>
+          <t>Each ticket has a ticket type: INCIDENT or SERVICE_REQUEST. ITIL foundational distinction. Promoted from SHOULD.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SHOULD</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -1865,10 +1865,76 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Auto-escalation on SLA breach — scheduled job reassigns to higher-tier agent + notifies management when SLA is at risk. System-driven.</t>
+          <t>Auto-escalation on SLA breach — two-stage (warning at 75%, reassign at 90%), per-company threshold via SLA_TARGETS.escalation_pct, workload-based agent selection, 5-min scheduler, hierarchical fallback when no higher tier. ITIL 4 + ISO 20000-1 §8.6.3 grounded.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>FR-36</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ITIL Alignment</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Resolution code + summary required on Resolve — records how it was resolved (FIXED, WORKAROUND, etc.) for trend analysis and future KB.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>FR-37</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ITIL Alignment</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Triage gate — priority required before moving to In Progress. Enforces ITIL categorization/prioritization step (page validation).</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>FR-38</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Comment notification — notify the other party when a comment is added (agent comments notify requester; client comments notify assigned agent).</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>SHOULD</t>
         </is>
@@ -2578,7 +2644,7 @@
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -2593,7 +2659,7 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -2619,7 +2685,7 @@
       </c>
       <c r="B7" s="13" t="n"/>
       <c r="C7" s="18" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add projects layer, role switching, new mockup pages + schema updates
Introduce PROJECTS table between COMPANIES and TICKETS (decision O),
USER_ROLES for multi-role switching (decision P), AGENT_PROJECTS and
USER_PROJECTS scoping. Add mockup pages 11/17/18, update schema/seed/views,
sync brief + all docs artifacts.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Ticketing-Requirements.xlsx
+++ b/docs/Ticketing-Requirements.xlsx
@@ -746,12 +746,12 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Auth &amp; Access</t>
+          <t>Authentication &amp; access</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>A client user only sees data belonging to their own company and department (tenant + dept isolation).</t>
+          <t>A client user only sees data belonging to their own company, scoped to projects they have access to (decision N/O). Default: all company projects (open). Client Admin can restrict via USER_PROJECTS. A Client Admin sees all company data across all projects.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -784,12 +784,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Companies &amp; Users</t>
+          <t>Companies &amp; users (admin)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>System Admin can create / edit / deactivate companies.</t>
+          <t>System Admin can create/edit/deactivate companies and projects (service engagements per company).</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -860,12 +860,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Tickets</t>
+          <t>Tickets - core</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>A client can raise a ticket (subject, description, category, severity). Severity (business impact) is client-set; Priority (work order) is support-set.</t>
+          <t>A client can raise a ticket (project, subject, description, category, severity). Client selects the project; if company has only one, it is auto-selected. Severity is client-set; Priority is support-set. Project, severity, and category are required at creation.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -974,12 +974,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Tickets</t>
+          <t>Tickets - core</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>A ticket can be assigned/reassigned. System Admin assigns anyone; clients assign from L1 agents mapped to their company; agents self-assign.</t>
+          <t>A ticket can be assigned/reassigned to a support agent. System Admin can assign any active agent; clients can assign from L1 agents only mapped to the ticket's project via AGENT_PROJECTS; Support Agents can self-assign from the open queue.</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -1164,12 +1164,12 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Find &amp; Filter</t>
+          <t>Finding &amp; filtering</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>See a list of permitted tickets, filterable by status, priority, severity, company, assignee. Includes ticket age column and SLA breach indicator.</t>
+          <t>Agents/admins can see a list of all tickets they're allowed to see, filterable by status, priority, severity, company, project, assignee. Includes ticket age and SLA breach indicator.</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1468,12 +1468,12 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>SLA &amp; Aging</t>
+          <t>SLA &amp; aging</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>SLA target per severity, per project (company) with breach highlighting — SLA_TARGETS keyed on (company_id, severity), colour-coded indicators.</t>
+          <t>SLA target per severity, per project with declarative breach highlighting. SLA_TARGETS maps project_id + severity to response_hours and resolution_days; sla_due_date stamped at creation.</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -1860,12 +1860,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SLA &amp; Aging</t>
+          <t>SLA &amp; aging</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Auto-escalation on SLA breach — two-stage (warning at 75%, reassign at 90%), per-company threshold via SLA_TARGETS.escalation_pct, workload-based agent selection, 5-min scheduler, hierarchical fallback when no higher tier. ITIL 4 + ISO 20000-1 §8.6.3 grounded.</t>
+          <t>Auto-escalation on SLA breach. Scheduled job (5-min interval) checks tickets against sla_due_date. Two-stage: warning at 75%, auto-reassign at 90% (within ticket's project). Per-project threshold via SLA_TARGETS.escalation_pct.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">

</xml_diff>

<commit_message>
docs: sync all artifacts at design lock — decisions M/P/Q/R/S propagated
Full /sync-docs run (deferral lifted at mockup lock-in):
- Brief: decision S landed (named SLA policies — SLA_POLICIES + SLA_TARGETS
  rekeyed to (sla_policy_id, severity), PROJECTS.sla_policy_id + globally
  unique company-prefixed project keys, one-door admin editing); FR-23/FR-35
  rewritten; data model now 13 tables
- HTML one-pager: FR texts, role cards, ERD (SLA_POLICIES, tier on
  AGENT_PROJECTS, USER_PROJECTS invitation list, PROJECTS.visibility),
  decision log A-S brought current, footer stamped design-locked
- XLSX: FR-4/5/6/7/10/23/26/35 texts updated
- PPTX slide 6: SLA line now "Named SLA policies"
- CLAUDE.md: roles, 13-table data model, isolation notes per decisions M/Q/S

verify: OK (MUST 18 / SHOULD 18 / COULD 2, 38 FRs)
</commit_message>
<xml_diff>
--- a/docs/Ticketing-Requirements.xlsx
+++ b/docs/Ticketing-Requirements.xlsx
@@ -746,12 +746,12 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Authentication &amp; access</t>
+          <t>Auth &amp; Access</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>A client user only sees data belonging to their own company, scoped to projects they have access to (decision N/O). Default: all company projects (open). Client Admin can restrict via USER_PROJECTS. A Client Admin sees all company data across all projects.</t>
+          <t>A client user only sees tickets from projects they can access: all Open projects of their company + invited Restricted projects (tenant + project isolation, decisions N/Q). Departments are metadata only.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -784,12 +784,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Companies &amp; users (admin)</t>
+          <t>Companies &amp; Users</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>System Admin can create/edit/deactivate companies and projects (service engagements per company).</t>
+          <t>System Admin can create/edit/deactivate companies and projects. Each project carries a visibility flag: OPEN (default, whole company sees it) or RESTRICTED (invitation-only, decision Q).</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>System Admin can create / edit / deactivate users and assign role + company.</t>
+          <t>System Admin can create/edit/deactivate users and assign role + company. Agent creation requires &gt;=1 AGENT_PROJECTS mapping, each carrying a tier (decision M revised); provider-company users auto-granted CLIENT_USER. Client Admin manages Restricted-project invitations.</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -860,12 +860,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Tickets - core</t>
+          <t>Tickets</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>A client can raise a ticket (project, subject, description, category, severity). Client selects the project; if company has only one, it is auto-selected. Severity is client-set; Priority is support-set. Project, severity, and category are required at creation.</t>
+          <t>A client can raise a ticket (project, subject, description, category, severity) - project auto-selected if the company has only one. Severity (business impact) is client-set; Priority (work order) is support-set.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -974,12 +974,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Tickets - core</t>
+          <t>Tickets</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>A ticket can be assigned/reassigned to a support agent. System Admin can assign any active agent; clients can assign from L1 agents only mapped to the ticket's project via AGENT_PROJECTS; Support Agents can self-assign from the open queue.</t>
+          <t>A ticket can be assigned/reassigned to a support agent. System Admin assigns anyone; clients assign from agents who are L1 on the ticket's project (tier per project, decisions J/L/M); agents self-assign.</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -1468,12 +1468,12 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>SLA &amp; aging</t>
+          <t>SLA &amp; Aging</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>SLA target per severity, per project with declarative breach highlighting. SLA_TARGETS maps project_id + severity to response_hours and resolution_days; sla_due_date stamped at creation.</t>
+          <t>Named SLA policies (Gold/Standard/Bronze/Internal, decision S) with per-severity targets + breach highlighting - SLA_POLICIES assigned via PROJECTS.sla_policy_id (is_default fallback), SLA_TARGETS keyed on (sla_policy_id, severity), colour-coded indicators.</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>A support agent/lead can reassign a ticket to a higher-tier agent (e.g. L1→L2) + optionally raise priority, written to history.</t>
+          <t>A support agent/lead can reassign a ticket to a same-or-higher-tier agent (e.g. L1-&gt;L2) + optionally raise priority, written to history. Tiers compared on the ticket's project (AGENT_PROJECTS, decision M revised).</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -1860,12 +1860,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SLA &amp; aging</t>
+          <t>SLA &amp; Aging</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Auto-escalation on SLA breach. Scheduled job (5-min interval) checks tickets against sla_due_date. Two-stage: warning at 75%, auto-reassign at 90% (within ticket's project). Per-project threshold via SLA_TARGETS.escalation_pct.</t>
+          <t>Auto-escalation on SLA breach - two-stage (warning at 75%, reassign at 90%), per-severity threshold via the policy's SLA_TARGETS.escalation_pct, next-tier agent read from AGENT_PROJECTS for the ticket's project, workload-based selection, 5-min scheduler, hierarchical fallback when no higher tier. ITIL 4 + ISO 20000-1 s8.6.3 grounded.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">

</xml_diff>

<commit_message>
docs: sync scope — 15 tables, FR-25 attachments built (MUST18/SHOULD19/COULD1)
- brief: FR-25 COULD->SHOULD (built 2026-07-05); ADMIN_AUDIT_LOG +
  TICKET_ATTACHMENTS in data model + ERD; AI (FR-24) stays COULD, blocked
  (every Generative AI provider needs an API key we don't have)
- HTML / XLSX / PPTX slide 6 / CLAUDE.md propagated; sync_docs verify = OK
</commit_message>
<xml_diff>
--- a/docs/Ticketing-Requirements.xlsx
+++ b/docs/Ticketing-Requirements.xlsx
@@ -1544,12 +1544,12 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Tickets - Stretch</t>
+          <t>Tickets</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>File / screenshot attachments on a ticket (proof/evidence); stored in TICKET_ATTACHMENTS, tenant-scoped (brief §5.1).</t>
+          <t>File / screenshot attachments on a ticket or comment (proof/evidence); stored in TICKET_ATTACHMENTS, tenant-scoped via V_MY_ATTACHMENTS. Built 2026-07-05 (promoted from COULD).</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>COULD</t>
+          <t>SHOULD</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -2659,7 +2659,7 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">

</xml_diff>